<commit_message>
feat: enrich system prompt with conversation_goal and preferred_musical_culture
Inject per-session conversation_goal (listener_goal) and user_profile
(preferred_musical_culture) into the LLM system prompt to improve
personalization and explanation quality for the LLM-Judge metric (30% weight).

- crs_baseline._get_system_prompt() now accepts conversation_goal and
  user_profile params; appends listener goal and musical culture to prompt
- run_inference_devset.py and run_inference_blindset.py extract and pass
  these fields from each dataset item
- Add docs on unused data opportunities (training data, embeddings)

🌀 Magic applied with Wibey VSCode Extension 🪄
</commit_message>
<xml_diff>
--- a/docs/leaderboard.xlsx
+++ b/docs/leaderboard.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/s0k0b3h/Workspace/03_Learn/RecSys_Baselines/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/s0k0b3h/Workspace/03_Learn/RecSys_Baselines/music-crs-baselines-main/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C586F4EC-07C8-E04C-B992-885A818C9CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{077080BF-3C16-2841-B6FA-6CEC54C8C732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2260" windowWidth="28040" windowHeight="17180" xr2:uid="{09145C04-5F8D-8D49-B5CA-1891E20BCA50}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Composite Score (Norm+Weighted)</t>
   </si>
@@ -66,6 +66,9 @@
   </si>
   <si>
     <t>Rank</t>
+  </si>
+  <si>
+    <t>SBert_Llama</t>
   </si>
 </sst>
 </file>
@@ -564,6 +567,26 @@
         <v>1.6</v>
       </c>
     </row>
+    <row r="4" spans="1:7" ht="20" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.13</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.04</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0.03</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.66</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1.55</v>
+      </c>
+    </row>
     <row r="6" spans="1:7" ht="21" x14ac:dyDescent="0.25">
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>

</xml_diff>